<commit_message>
Add verified Ebola response coverage
Add UNICEF EOC 2018-2019 and INSP/INRB 2026 Ebola response records to all RFO workbooks, update source and validation documentation, and expose the new coverage in the public map and landing page.\n\nCo-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mambasa_Humanitarian_3W_Matrix.xlsx
+++ b/Mambasa_Humanitarian_3W_Matrix.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="5Ws MODEL" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="4Ws MODEL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="5Ws Guide" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="5Ws Database" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="RFO STAKEHOLDER" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="RFO STAKEHOLDER HISTORY" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Coverage Summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Data Notes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Data Sources" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Historical Coverage" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="3W Matrix (Who does What Where)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Cluster Summary (Who Does What)" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="WorldPop Estimates" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5Ws MODEL" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4Ws MODEL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5Ws Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5Ws Database" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFO STAKEHOLDER" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFO STAKEHOLDER HISTORY" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Coverage" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3W Matrix (Who does What Where)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster Summary (Who Does What)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorldPop Estimates" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'5Ws MODEL'!$A$1:$V$154</definedName>
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB154"/>
+  <dimension ref="A1:AB164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19782,6 +19782,1426 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-001</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>Ebola case surveillance and line-list reporting in Mandima Health Zone</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>Support outbreak surveillance, case investigation and response coordination in an affected health zone</t>
+        </is>
+      </c>
+      <c r="G155" s="14" t="inlineStr">
+        <is>
+          <t>2018-08-05</t>
+        </is>
+      </c>
+      <c r="H155" s="14" t="inlineStr">
+        <is>
+          <t>2019-08-05</t>
+        </is>
+      </c>
+      <c r="I155" s="5" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="J155" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K155" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L155" s="5" t="inlineStr">
+        <is>
+          <t>Mandima</t>
+        </is>
+      </c>
+      <c r="M155" s="5" t="inlineStr">
+        <is>
+          <t>Mandima Health Zone</t>
+        </is>
+      </c>
+      <c r="N155" s="5" t="inlineStr">
+        <is>
+          <t>0.87° N, 29.75° E</t>
+        </is>
+      </c>
+      <c r="O155" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P155" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q155" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R155" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S155" s="5" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="T155" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF EOC annual dashboard: 238 Mandima line-list records (234 confirmed, 4 probable); health-zone geography used as Mambasa Territory proxy</t>
+        </is>
+      </c>
+      <c r="U155" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; territory assignment requires validation</t>
+        </is>
+      </c>
+      <c r="V155" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/unicef-eoc-2018-2019-dashboard-en-final</t>
+        </is>
+      </c>
+      <c r="W155" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X155" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y155" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z155" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA155" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB155" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-002</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>Ebola case investigation and line-list reporting in Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>Detect, investigate and refer suspected and confirmed Ebola cases</t>
+        </is>
+      </c>
+      <c r="G156" s="14" t="inlineStr">
+        <is>
+          <t>2019-07-09</t>
+        </is>
+      </c>
+      <c r="H156" s="14" t="inlineStr">
+        <is>
+          <t>2019-08-05</t>
+        </is>
+      </c>
+      <c r="I156" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="J156" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K156" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L156" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="M156" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="N156" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="O156" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P156" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q156" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R156" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S156" s="5" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="T156" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF EOC annual dashboard records 9 confirmed Mambasa-zone cases; health-zone geography used as territory proxy</t>
+        </is>
+      </c>
+      <c r="U156" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; case counts are not beneficiary counts</t>
+        </is>
+      </c>
+      <c r="V156" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/unicef-eoc-2018-2019-dashboard-en-final</t>
+        </is>
+      </c>
+      <c r="W156" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X156" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y156" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z156" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA156" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB156" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-003</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Psychosocial and protection</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>Psychosocial support, child protection and family support during Ebola response</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>Reduce psychosocial harm and protect children and families affected by Ebola</t>
+        </is>
+      </c>
+      <c r="G157" s="14" t="inlineStr">
+        <is>
+          <t>2019-04-01</t>
+        </is>
+      </c>
+      <c r="H157" s="14" t="inlineStr">
+        <is>
+          <t>2019-04-30</t>
+        </is>
+      </c>
+      <c r="I157" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="J157" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K157" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L157" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa / Mandima</t>
+        </is>
+      </c>
+      <c r="M157" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa and Mandima Health Zones</t>
+        </is>
+      </c>
+      <c r="N157" s="5" t="inlineStr">
+        <is>
+          <t>1.21° N, 28.48° E</t>
+        </is>
+      </c>
+      <c r="O157" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P157" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q157" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R157" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S157" s="5" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="T157" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF April 2019 psychosocial pillar database records CTE/CT support, psychoeducation and family assistance in both health zones</t>
+        </is>
+      </c>
+      <c r="U157" s="5" t="inlineStr">
+        <is>
+          <t>Approximate combined health-zone reference; validate locality-specific coverage</t>
+        </is>
+      </c>
+      <c r="V157" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/ebola-unicef-eoc-psychosocial-pillar-database-drc-april-2019</t>
+        </is>
+      </c>
+      <c r="W157" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X157" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y157" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z157" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA157" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB157" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-004</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Psychosocial, protection and nutrition</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>Psychosocial support, separated-child assistance and nutrition support</t>
+        </is>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>Protect children and provide family and nutrition support during Ebola response</t>
+        </is>
+      </c>
+      <c r="G158" s="14" t="inlineStr">
+        <is>
+          <t>2019-05-01</t>
+        </is>
+      </c>
+      <c r="H158" s="14" t="inlineStr">
+        <is>
+          <t>2019-05-31</t>
+        </is>
+      </c>
+      <c r="I158" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="J158" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K158" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L158" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa / Mandima</t>
+        </is>
+      </c>
+      <c r="M158" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa and Mandima Health Zones</t>
+        </is>
+      </c>
+      <c r="N158" s="5" t="inlineStr">
+        <is>
+          <t>1.21° N, 28.48° E</t>
+        </is>
+      </c>
+      <c r="O158" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P158" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q158" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R158" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S158" s="5" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="T158" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF May 2019 psychosocial database records CTE support, contact/family follow-up and food/nutrition kit distribution in both zones</t>
+        </is>
+      </c>
+      <c r="U158" s="5" t="inlineStr">
+        <is>
+          <t>Approximate combined health-zone reference; validate locality-specific coverage</t>
+        </is>
+      </c>
+      <c r="V158" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/unicef-eoc-psychosocial-mai-2019-dataset</t>
+        </is>
+      </c>
+      <c r="W158" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X158" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y158" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z158" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA158" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB158" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-005</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Psychosocial and protection</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>Psychosocial support, contact/family follow-up and child protection</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>Support affected people, contacts, families and children during outbreak response</t>
+        </is>
+      </c>
+      <c r="G159" s="14" t="inlineStr">
+        <is>
+          <t>2019-06-01</t>
+        </is>
+      </c>
+      <c r="H159" s="14" t="inlineStr">
+        <is>
+          <t>2019-06-30</t>
+        </is>
+      </c>
+      <c r="I159" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K159" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L159" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa / Mandima</t>
+        </is>
+      </c>
+      <c r="M159" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa and Mandima Health Zones</t>
+        </is>
+      </c>
+      <c r="N159" s="5" t="inlineStr">
+        <is>
+          <t>1.21° N, 28.48° E</t>
+        </is>
+      </c>
+      <c r="O159" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P159" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q159" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R159" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S159" s="5" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="T159" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF June 2019 psychosocial database records support for suspected/confirmed cases, contacts, families and children</t>
+        </is>
+      </c>
+      <c r="U159" s="5" t="inlineStr">
+        <is>
+          <t>Approximate combined health-zone reference; validate locality-specific coverage</t>
+        </is>
+      </c>
+      <c r="V159" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/unicef-eoc-psychosocial-juin-2019-dataset</t>
+        </is>
+      </c>
+      <c r="W159" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X159" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y159" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z159" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA159" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB159" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-001</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>INSP / INRB BDBV response</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>Routine surveillance, alerts, investigations, active case finding and contact follow-up</t>
+        </is>
+      </c>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>Detect and contain suspected Bundibugyo virus transmission in Mambasa</t>
+        </is>
+      </c>
+      <c r="G160" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="H160" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J160" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K160" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L160" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="M160" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="N160" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="O160" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P160" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q160" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R160" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S160" s="5" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="T160" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB public response monitoring records surveillance and investigations in Mambasa; preliminary sitrep-derived data</t>
+        </is>
+      </c>
+      <c r="U160" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; BDBV records require routine official validation</t>
+        </is>
+      </c>
+      <c r="V160" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data/blob/main/data/public_health_response/processed/public_health_response__epidemiological_monitoring_en__daily.csv</t>
+        </is>
+      </c>
+      <c r="W160" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X160" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y160" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z160" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA160" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB160" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-002</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>INSP / INRB BDBV response</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Infection prevention and control</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>IPC briefings, WASH and IPC kit distribution for Mambasa providers</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>Reduce healthcare-associated transmission through IPC and WASH readiness</t>
+        </is>
+      </c>
+      <c r="G161" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="H161" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="I161" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J161" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K161" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L161" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="M161" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="N161" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="O161" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P161" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q161" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R161" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S161" s="5" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="T161" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB public response monitoring records provider briefings and IPC/WASH kit support in Mambasa</t>
+        </is>
+      </c>
+      <c r="U161" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; BDBV records are preliminary</t>
+        </is>
+      </c>
+      <c r="V161" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data/blob/main/data/public_health_response/processed/public_health_response__epidemiological_infection_prevention_controle_en__daily.csv</t>
+        </is>
+      </c>
+      <c r="W161" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X161" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y161" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z161" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA161" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB161" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-003</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>INSP / INRB BDBV response</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Points of control and laboratory preparedness</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>Activation of points of control, referrals and laboratory preparedness</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>Strengthen early detection, referral and diagnostic readiness in Mambasa</t>
+        </is>
+      </c>
+      <c r="G162" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="H162" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="I162" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J162" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="K162" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="L162" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="M162" s="5" t="inlineStr">
+        <is>
+          <t>Mabake / Mambasa points of control and Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="N162" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="O162" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P162" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q162" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R162" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S162" s="5" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="T162" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB provincial monitoring records PoC activation, referrals and laboratory installations; WHO-supported supplies are noted in logistics records</t>
+        </is>
+      </c>
+      <c r="U162" s="5" t="inlineStr">
+        <is>
+          <t>Approximate operational reference; names and boundaries require partner validation</t>
+        </is>
+      </c>
+      <c r="V162" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data/blob/main/data/public_health_response/processed/public_health_response__provincial_epidemiological_monitoring_en__daily.csv</t>
+        </is>
+      </c>
+      <c r="W162" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X162" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y162" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z162" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA162" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB162" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-004</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>INSP / DRC public health response</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>BDBV case surveillance and cumulative case/death monitoring</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>Monitor and coordinate response to confirmed Bundibugyo virus transmission in Wamba</t>
+        </is>
+      </c>
+      <c r="G163" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="H163" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="I163" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>Haut-Uele</t>
+        </is>
+      </c>
+      <c r="K163" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="L163" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="M163" s="5" t="inlineStr">
+        <is>
+          <t>Wamba Health Zone</t>
+        </is>
+      </c>
+      <c r="N163" s="5" t="inlineStr">
+        <is>
+          <t>2.14° N, 27.99° E</t>
+        </is>
+      </c>
+      <c r="O163" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P163" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q163" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R163" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S163" s="5" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="T163" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB-derived cumulative series reports Wamba first confirmed case on 10 July and 83 confirmed cases/31 deaths by 5 September; preliminary data</t>
+        </is>
+      </c>
+      <c r="U163" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; epidemiological data require official validation</t>
+        </is>
+      </c>
+      <c r="V163" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data/blob/main/data/insp_sitrep/processed/insp_sitrep__cumulative_confirmed_cases__daily.csv</t>
+        </is>
+      </c>
+      <c r="W163" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X163" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y163" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z163" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA163" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB163" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-005</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>INSP / DRC public health response</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Community engagement</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>Community communication around confirmed Wamba cases</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>Improve risk awareness and promote timely care-seeking and prevention</t>
+        </is>
+      </c>
+      <c r="G164" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H164" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="I164" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J164" s="5" t="inlineStr">
+        <is>
+          <t>Haut-Uele</t>
+        </is>
+      </c>
+      <c r="K164" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="L164" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="M164" s="5" t="inlineStr">
+        <is>
+          <t>Wamba Health Zone</t>
+        </is>
+      </c>
+      <c r="N164" s="5" t="inlineStr">
+        <is>
+          <t>2.14° N, 27.99° E</t>
+        </is>
+      </c>
+      <c r="O164" s="5" t="inlineStr">
+        <is>
+          <t>3,705 people reached</t>
+        </is>
+      </c>
+      <c r="P164" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q164" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="R164" s="5" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="S164" s="5" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="T164" s="5" t="inlineStr">
+        <is>
+          <t>National INSP sitrep records community communication reaching 3,705 people in Wamba; implementing partner not specified</t>
+        </is>
+      </c>
+      <c r="U164" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; reach figure is not a unique beneficiary count</t>
+        </is>
+      </c>
+      <c r="V164" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data/blob/main/data/public_health_response/processed/public_health_response__national_epidemiological_community_engagement_en__daily.csv</t>
+        </is>
+      </c>
+      <c r="W164" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="X164" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Y164" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="Z164" s="5" t="inlineStr">
+        <is>
+          <t>Not calculated</t>
+        </is>
+      </c>
+      <c r="AA164" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response record; beneficiary estimate not calculated</t>
+        </is>
+      </c>
+      <c r="AB164" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable for response activity record</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V154"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19797,7 +21217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19962,6 +21382,33 @@
       <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Latest workbook date; not a new source reporting period</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2018-2026 Ebola response</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UNICEF EOC historical datasets and INSP/INRB BDBV public monitoring</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>9 source-backed 5Ws records</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mambasa (Mambasa/Mandima health zones) and Wamba; no Watsa-specific verified record</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Health-zone geography is a proxy; 2026 BDBV data are preliminary and require partner/government validation</t>
         </is>
       </c>
     </row>
@@ -38807,7 +40254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T154"/>
+  <dimension ref="A1:T164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -52653,6 +54100,1026 @@
       <c r="T154" s="5" t="inlineStr">
         <is>
           <t>Reference coordinate; not verified facility-level GPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-001</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>Ebola case surveillance and line-list reporting in Mandima Health Zone</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H155" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I155" s="5" t="inlineStr">
+        <is>
+          <t>Mandima</t>
+        </is>
+      </c>
+      <c r="J155" s="5" t="inlineStr">
+        <is>
+          <t>Mandima Health Zone</t>
+        </is>
+      </c>
+      <c r="K155" s="5" t="inlineStr">
+        <is>
+          <t>0.87° N, 29.75° E</t>
+        </is>
+      </c>
+      <c r="L155" s="12" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="M155" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF EOC annual dashboard: 238 Mandima line-list records (234 confirmed, 4 probable); health-zone geography used as Mambasa Territory proxy</t>
+        </is>
+      </c>
+      <c r="N155" s="10" t="inlineStr">
+        <is>
+          <t>2018-08-05</t>
+        </is>
+      </c>
+      <c r="O155" s="10" t="inlineStr">
+        <is>
+          <t>2019-08-05</t>
+        </is>
+      </c>
+      <c r="P155" s="5" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="Q155" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R155" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/a3fe7795-dbe3-410f-942c-ef407c040868/resource/deaa1018-df33-4b92-8afc-c67f0b2c0fea/download/annual-dashboard-unicef-eoc.xlsx</t>
+        </is>
+      </c>
+      <c r="S155" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; territory assignment requires validation</t>
+        </is>
+      </c>
+      <c r="T155" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF EOC annual dashboard: 238 Mandima line-list records (234 confirmed, 4 probable); health-zone geography used as Mambasa Territory proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-002</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>Ebola case investigation and line-list reporting in Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="G156" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H156" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I156" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="J156" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="K156" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="L156" s="12" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="M156" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF EOC annual dashboard records 9 confirmed Mambasa-zone cases; health-zone geography used as territory proxy</t>
+        </is>
+      </c>
+      <c r="N156" s="10" t="inlineStr">
+        <is>
+          <t>2019-07-09</t>
+        </is>
+      </c>
+      <c r="O156" s="10" t="inlineStr">
+        <is>
+          <t>2019-08-05</t>
+        </is>
+      </c>
+      <c r="P156" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="Q156" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R156" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/a3fe7795-dbe3-410f-942c-ef407c040868/resource/deaa1018-df33-4b92-8afc-c67f0b2c0fea/download/annual-dashboard-unicef-eoc.xlsx</t>
+        </is>
+      </c>
+      <c r="S156" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; case counts are not beneficiary counts</t>
+        </is>
+      </c>
+      <c r="T156" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF EOC annual dashboard records 9 confirmed Mambasa-zone cases; health-zone geography used as territory proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-003</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Psychosocial and protection</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>Psychosocial support, child protection and family support during Ebola response</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H157" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I157" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa / Mandima</t>
+        </is>
+      </c>
+      <c r="J157" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa and Mandima Health Zones</t>
+        </is>
+      </c>
+      <c r="K157" s="5" t="inlineStr">
+        <is>
+          <t>1.21° N, 28.48° E</t>
+        </is>
+      </c>
+      <c r="L157" s="12" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="M157" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF April 2019 psychosocial pillar database records CTE/CT support, psychoeducation and family assistance in both health zones</t>
+        </is>
+      </c>
+      <c r="N157" s="10" t="inlineStr">
+        <is>
+          <t>2019-04-01</t>
+        </is>
+      </c>
+      <c r="O157" s="10" t="inlineStr">
+        <is>
+          <t>2019-04-30</t>
+        </is>
+      </c>
+      <c r="P157" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="Q157" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R157" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/b554c216-ab2e-4065-bc17-918f215bea86/resource/e4825dff-2410-4cfe-bb42-4a2b1d43ca02/download/psychosocial-avril-2019-unicef-eoc.xls</t>
+        </is>
+      </c>
+      <c r="S157" s="5" t="inlineStr">
+        <is>
+          <t>Approximate combined health-zone reference; validate locality-specific coverage</t>
+        </is>
+      </c>
+      <c r="T157" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF April 2019 psychosocial pillar database records CTE/CT support, psychoeducation and family assistance in both health zones</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-004</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Psychosocial, protection and nutrition</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>Psychosocial support, separated-child assistance and nutrition support</t>
+        </is>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="G158" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H158" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I158" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa / Mandima</t>
+        </is>
+      </c>
+      <c r="J158" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa and Mandima Health Zones</t>
+        </is>
+      </c>
+      <c r="K158" s="5" t="inlineStr">
+        <is>
+          <t>1.21° N, 28.48° E</t>
+        </is>
+      </c>
+      <c r="L158" s="12" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="M158" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF May 2019 psychosocial database records CTE support, contact/family follow-up and food/nutrition kit distribution in both zones</t>
+        </is>
+      </c>
+      <c r="N158" s="10" t="inlineStr">
+        <is>
+          <t>2019-05-01</t>
+        </is>
+      </c>
+      <c r="O158" s="10" t="inlineStr">
+        <is>
+          <t>2019-05-31</t>
+        </is>
+      </c>
+      <c r="P158" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="Q158" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R158" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/d047e4be-091f-4afb-b677-c964262a3cc3/resource/0716d640-20b3-4ff7-a3cb-3eea0cb5a933/download/unicef-ebola-master_psychosocial_mai-2019.xls</t>
+        </is>
+      </c>
+      <c r="S158" s="5" t="inlineStr">
+        <is>
+          <t>Approximate combined health-zone reference; validate locality-specific coverage</t>
+        </is>
+      </c>
+      <c r="T158" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF May 2019 psychosocial database records CTE support, contact/family follow-up and food/nutrition kit distribution in both zones</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>EB-2019-005</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>UN agency</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Psychosocial and protection</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>Psychosocial support, contact/family follow-up and child protection</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H159" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I159" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa / Mandima</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa and Mandima Health Zones</t>
+        </is>
+      </c>
+      <c r="K159" s="5" t="inlineStr">
+        <is>
+          <t>1.21° N, 28.48° E</t>
+        </is>
+      </c>
+      <c r="L159" s="12" t="inlineStr">
+        <is>
+          <t>Historical verified</t>
+        </is>
+      </c>
+      <c r="M159" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF June 2019 psychosocial database records support for suspected/confirmed cases, contacts, families and children</t>
+        </is>
+      </c>
+      <c r="N159" s="10" t="inlineStr">
+        <is>
+          <t>2019-06-01</t>
+        </is>
+      </c>
+      <c r="O159" s="10" t="inlineStr">
+        <is>
+          <t>2019-06-30</t>
+        </is>
+      </c>
+      <c r="P159" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="Q159" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R159" s="5" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/ec6827e1-e83b-4854-852e-a7c710f1685f/resource/81b3d06a-907d-4ed1-bb70-b02bd709cb64/download/unicef-ebola-master_psychosocial_juin-2019.xls</t>
+        </is>
+      </c>
+      <c r="S159" s="5" t="inlineStr">
+        <is>
+          <t>Approximate combined health-zone reference; validate locality-specific coverage</t>
+        </is>
+      </c>
+      <c r="T159" s="5" t="inlineStr">
+        <is>
+          <t>UNICEF June 2019 psychosocial database records support for suspected/confirmed cases, contacts, families and children</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-001</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>INSP / INRB BDBV response</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>Routine surveillance, alerts, investigations, active case finding and contact follow-up</t>
+        </is>
+      </c>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G160" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H160" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="J160" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="K160" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="L160" s="12" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="M160" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB public response monitoring records surveillance and investigations in Mambasa; preliminary sitrep-derived data</t>
+        </is>
+      </c>
+      <c r="N160" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="O160" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="P160" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q160" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R160" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data</t>
+        </is>
+      </c>
+      <c r="S160" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; BDBV records require routine official validation</t>
+        </is>
+      </c>
+      <c r="T160" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB public response monitoring records surveillance and investigations in Mambasa; preliminary sitrep-derived data</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-002</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>INSP / INRB BDBV response</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Infection prevention and control</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>IPC briefings, WASH and IPC kit distribution for Mambasa providers</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H161" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I161" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="J161" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="K161" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="L161" s="12" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="M161" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB public response monitoring records provider briefings and IPC/WASH kit support in Mambasa</t>
+        </is>
+      </c>
+      <c r="N161" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="O161" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="P161" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q161" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R161" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data</t>
+        </is>
+      </c>
+      <c r="S161" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; BDBV records are preliminary</t>
+        </is>
+      </c>
+      <c r="T161" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB public response monitoring records provider briefings and IPC/WASH kit support in Mambasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-003</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>INSP / INRB BDBV response</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Points of control and laboratory preparedness</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>Activation of points of control, referrals and laboratory preparedness</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G162" s="5" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="H162" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="I162" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="J162" s="5" t="inlineStr">
+        <is>
+          <t>Mabake / Mambasa points of control and Mambasa Health Zone</t>
+        </is>
+      </c>
+      <c r="K162" s="5" t="inlineStr">
+        <is>
+          <t>1.55° N, 27.20° E</t>
+        </is>
+      </c>
+      <c r="L162" s="12" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="M162" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB provincial monitoring records PoC activation, referrals and laboratory installations; WHO-supported supplies are noted in logistics records</t>
+        </is>
+      </c>
+      <c r="N162" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="O162" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="P162" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q162" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R162" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data</t>
+        </is>
+      </c>
+      <c r="S162" s="5" t="inlineStr">
+        <is>
+          <t>Approximate operational reference; names and boundaries require partner validation</t>
+        </is>
+      </c>
+      <c r="T162" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB provincial monitoring records PoC activation, referrals and laboratory installations; WHO-supported supplies are noted in logistics records</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-004</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>INSP / DRC public health response</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Surveillance</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>BDBV case surveillance and cumulative case/death monitoring</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G163" s="5" t="inlineStr">
+        <is>
+          <t>Haut-Uele</t>
+        </is>
+      </c>
+      <c r="H163" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="I163" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>Wamba Health Zone</t>
+        </is>
+      </c>
+      <c r="K163" s="5" t="inlineStr">
+        <is>
+          <t>2.14° N, 27.99° E</t>
+        </is>
+      </c>
+      <c r="L163" s="12" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="M163" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB-derived cumulative series reports Wamba first confirmed case on 10 July and 83 confirmed cases/31 deaths by 5 September; preliminary data</t>
+        </is>
+      </c>
+      <c r="N163" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="O163" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="P163" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q163" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R163" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data</t>
+        </is>
+      </c>
+      <c r="S163" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; epidemiological data require official validation</t>
+        </is>
+      </c>
+      <c r="T163" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB-derived cumulative series reports Wamba first confirmed case on 10 July and 83 confirmed cases/31 deaths by 5 September; preliminary data</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>EB-2026-005</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>INSP / DRC public health response</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response / Community engagement</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>Community communication around confirmed Wamba cases</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G164" s="5" t="inlineStr">
+        <is>
+          <t>Haut-Uele</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="I164" s="5" t="inlineStr">
+        <is>
+          <t>Wamba</t>
+        </is>
+      </c>
+      <c r="J164" s="5" t="inlineStr">
+        <is>
+          <t>Wamba Health Zone</t>
+        </is>
+      </c>
+      <c r="K164" s="5" t="inlineStr">
+        <is>
+          <t>2.14° N, 27.99° E</t>
+        </is>
+      </c>
+      <c r="L164" s="12" t="inlineStr">
+        <is>
+          <t>Current preliminary</t>
+        </is>
+      </c>
+      <c r="M164" s="5" t="inlineStr">
+        <is>
+          <t>National INSP sitrep records community communication reaching 3,705 people in Wamba; implementing partner not specified</t>
+        </is>
+      </c>
+      <c r="N164" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="O164" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="P164" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q164" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC / INSP-INRB BDBV</t>
+        </is>
+      </c>
+      <c r="R164" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data</t>
+        </is>
+      </c>
+      <c r="S164" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone reference; reach figure is not a unique beneficiary count</t>
+        </is>
+      </c>
+      <c r="T164" s="5" t="inlineStr">
+        <is>
+          <t>National INSP sitrep records community communication reaching 3,705 people in Wamba; implementing partner not specified</t>
         </is>
       </c>
     </row>
@@ -56906,7 +59373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -57198,6 +59665,42 @@
       <c r="B24" t="inlineStr">
         <is>
           <t>Validate locality coordinates, boundaries and intervention targets with partners before reporting. Do not aggregate rows across interventions without deduplicating people reached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ebola response records</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Verified historical UNICEF EOC records cover Mambasa and Mandima Health Zones during the 2018-2019 North Kivu/Ituri Ebola outbreak. Preliminary INSP/INRB BDBV monitoring records cover Mambasa in June-July 2026 and Wamba in July-September 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Ebola geographic limitation</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Health zones are used as operational geography proxies for territory-level reporting. Watsa has no verified Ebola-specific operation in the reviewed public sources; this is an evidence gap, not proof of no activity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ebola beneficiary limitation</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Ebola case counts, people reached and response outputs are not interchangeable with unique beneficiaries. They remain in source/verification fields and are not added to WorldPop intervention estimates.</t>
         </is>
       </c>
     </row>
@@ -57212,7 +59715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -57383,6 +59886,38 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ebola response evidence: UNICEF EOC and INSP/INRB BDBV public data</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UNICEF EOC; DRC Ministry of Health/INSP/INRB; WHO-supported response</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Historical 2018-2019 Ebola response records in Mambasa/Mandima health zones and preliminary 2026 BDBV response records in Mambasa and Wamba; no verified Watsa-specific operation identified</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2019 historical extracts and 2026 preliminary public monitoring data</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/unicef-eoc-2018-2019-dashboard-en-final; https://github.com/INRB-UMIE/BDBV2026-Data</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ebola response activities, surveillance, psychosocial support, IPC, points of control, laboratory readiness and community engagement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Ebola response organisations register
Add a source-backed Ebola Organisations sheet and align the stakeholder registers with Ebola response roles, periods, locations, and validation status across all RFO workbooks.\n\nCo-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mambasa_Humanitarian_3W_Matrix.xlsx
+++ b/Mambasa_Humanitarian_3W_Matrix.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3W Matrix (Who does What Where)" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster Summary (Who Does What)" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorldPop Estimates" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ebola Organisations" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'5Ws MODEL'!$A$1:$V$154</definedName>
@@ -29,6 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Coverage Summary'!$A$1:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Data Sources'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Historical Coverage'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Ebola Organisations'!$A$1:$I$11</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +61,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -103,6 +105,11 @@
         <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B1F33"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -141,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,6 +194,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -25152,6 +25162,549 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Actor Type</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
+        <is>
+          <t>Province(s)</t>
+        </is>
+      </c>
+      <c r="D1" s="16" t="inlineStr">
+        <is>
+          <t>Territory(ies)</t>
+        </is>
+      </c>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>Ebola response role / sector</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>Operation years</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>Evidence and geographic note</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>Verification status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>INSP / INRB</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Government / public health institute</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Ituri; Haut-Uele</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa; Wamba</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Surveillance, IPC/WASH, points of control, laboratory preparedness, community engagement</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa and Wamba records are preliminary BDBV monitoring data; verify with official response coordination</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>https://github.com/INRB-UMIE/BDBV2026-Data</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>Verified public-source response actor; preliminary data</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>UNICEF Ebola Emergency Operations Centre</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>UN agency / response coordination</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Surveillance, psychosocial support, child protection, nutrition and family support</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>UNICEF EOC dashboards and psychosocial pillar datasets document Mambasa and Mandima health-zone activities</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/unicef-eoc-2018-2019-dashboard-en-final</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>Verified public-source response actor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>DRC Ministry of Health</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Government / public health</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Ituri; Haut-Uele</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa; Wamba</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Ebola/BDBV response leadership, surveillance, case management and coordination</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019; 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Named as the national response authority in UNICEF, CDC and INSP/INRB public response sources; territory-level implementing detail requires validation</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/68/wr/mm6850a3.htm</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Response authority; territory-level activity requires validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>WHO</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>UN agency / technical partner</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Ituri; Haut-Uele</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa; Wamba</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Technical support, emergency mapping, IPC, logistics and response coordination</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019; 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>WHO is identified in Ebola response sources and WHO-supported 2026 logistics records; exact organisation-level outputs require validation</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>https://data.humdata.org/dataset/drc-health-facilities</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Provincial/national response partner; local outputs require validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>OCHA</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>UN agency / coordination</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Ituri; Haut-Uele</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa; Wamba</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Humanitarian coordination and response information management</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>CDC response context identifies OCHA among response partners; no locality-specific activity count asserted</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/68/wr/mm6850a3.htm</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Provincial/national response partner; local outputs require validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>UN agency / humanitarian partner</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Humanitarian coordination, displacement and response support</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>CDC response context identifies IOM among response partners; no locality-specific activity count asserted</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/68/wr/mm6850a3.htm</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>Provincial/national response partner; local outputs require validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>ALIMA</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>International NGO / medical response partner</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Case management, treatment and emergency medical response</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>CDC response context identifies ALIMA among response partners; exact Mambasa activity requires partner validation</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/68/wr/mm6850a3.htm</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Provincial/national response partner; local outputs require validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Médecins Sans Frontières (MSF)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>International NGO / medical response partner</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Ituri; Haut-Uele</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa; Wamba</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Case management, IPC and emergency health response</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019; 2026</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>MSF is an existing stakeholder and is named in CDC response context; Ebola-specific local outputs require validation</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/68/wr/mm6850a3.htm</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Existing stakeholder; Ebola role requires local validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Croix-Rouge de la RDC</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>National NGO / response partner</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Ituri; Haut-Uele</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa; Wamba</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Community engagement, surveillance and emergency response support</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019; 2026</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Existing stakeholder named in CDC response context; Ebola-specific local outputs require validation</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/68/wr/mm6850a3.htm</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>Existing stakeholder; Ebola role requires local validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>CDC</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Government technical partner</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Ituri</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Mambasa</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Technical assistance, surveillance and outbreak response support</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>2018-2019</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>CDC published response context for the North Kivu/Ituri Ebola outbreak; no locality-specific activity count asserted</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/mmwr/volumes/68/wr/mm6850a3.htm</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Technical response partner; local outputs require validation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -55138,7 +55691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -57666,7 +58219,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Protection, WASH</t>
+          <t>Protection, WASH; Ebola response</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
@@ -57676,12 +58229,12 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026; 2018-2019; 2026</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Biakato, Ibambi, Mambasa Centre, Pawa, Wamba Centre</t>
+          <t>Biakato, Ibambi, Mambasa Centre, Pawa, Wamba Centre; Mambasa, Mandima, Wamba</t>
         </is>
       </c>
       <c r="I26" s="5" t="n">
@@ -57734,12 +58287,12 @@
       </c>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>No budget total published; validate with partner</t>
+          <t>No budget total published; validate with partner; Ebola role source-backed; exact local outputs require validation</t>
         </is>
       </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>Mambasa Humanitarian workbook - à valider</t>
+          <t>Mambasa Humanitarian workbook - à valider; UNICEF EOC Ebola datasets; INSP/INRB BDBV2026 public data</t>
         </is>
       </c>
     </row>
@@ -58040,6 +58593,88 @@
       <c r="T29" s="5" t="inlineStr">
         <is>
           <t>Mambasa Humanitarian workbook - à valider</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>INSP / INRB</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Government / public health institute</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Ituri; Haut-Uele</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa; Wamba</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Ebola response: surveillance, IPC/WASH, points of control, laboratory preparedness, community engagement</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Detect and contain Bundibugyo virus transmission and maintain public-health readiness</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Mambasa Health Zone; Wamba Health Zone</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>10 Ebola response records</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Approximate health-zone references</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Mambasa 1.55° N, 27.20° E; Wamba 2.14° N, 27.99° E</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Health-zone proxy; validate exact operational sites</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="5" t="n"/>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>Response outputs and case data are not unique beneficiary counts</t>
+        </is>
+      </c>
+      <c r="P30" s="5" t="n"/>
+      <c r="Q30" s="5" t="n"/>
+      <c r="R30" s="5" t="n"/>
+      <c r="S30" s="5" t="inlineStr">
+        <is>
+          <t>Preliminary public INSP/INRB data; validate with response coordination</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="inlineStr">
+        <is>
+          <t>INSP/INRB BDBV2026 public data</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Ebola response funding data
Add OCHA FTS funding flows and 2026 BDBV funding-status records, enrich Ebola organisation funding fields, and document geographic attribution limits across the RFO workbooks.\n\nCo-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mambasa_Humanitarian_3W_Matrix.xlsx
+++ b/Mambasa_Humanitarian_3W_Matrix.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster Summary (Who Does What)" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorldPop Estimates" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ebola Organisations" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ebola Funding" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'5Ws MODEL'!$A$1:$V$154</definedName>
@@ -31,6 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Data Sources'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Historical Coverage'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Ebola Organisations'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Ebola Funding'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -25168,7 +25170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -25228,6 +25230,21 @@
           <t>Verification status</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Funding source(s) / published amount</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Funding geographic scope</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Funding QA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -25275,6 +25292,21 @@
           <t>Verified public-source response actor; preliminary data</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Not publicly published</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mambasa/Wamba local funding not published</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>No public donor or amount identified</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -25322,6 +25354,21 @@
           <t>Verified public-source response actor</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CERF US$3,935,937; ECHO US$889,878 (2019)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Source-backed provincial funding; local attribution unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -25369,6 +25416,21 @@
           <t>Response authority; territory-level activity requires validation</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Not separately published</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>National/provincial response authority</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>No ministry-specific amount identified</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -25416,6 +25478,21 @@
           <t>Provincial/national response partner; local outputs require validation</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CERF US$1,701,255 (2018); CERF US$3,902,590 (2019); ECHO US$8,476,085; Germany US$7,786,429</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Source-backed provincial funding; local attribution unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -25463,6 +25540,21 @@
           <t>Provincial/national response partner; local outputs require validation</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Not separately published</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Response-wide/provincial context only</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>No organisation-specific amount identified</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -25510,6 +25602,21 @@
           <t>Provincial/national response partner; local outputs require validation</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>CERF US$1,999,062 (2019)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Source-backed provincial funding; local attribution unavailable</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -25557,6 +25664,21 @@
           <t>Provincial/national response partner; local outputs require validation</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Not separately published in reviewed FTS records</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Provincial response context only</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>No organisation-specific amount identified</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -25604,6 +25726,21 @@
           <t>Existing stakeholder; Ebola role requires local validation</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Not separately published in reviewed FTS records</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Provincial response context only</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>No organisation-specific amount identified</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -25651,6 +25788,21 @@
           <t>Existing stakeholder; Ebola role requires local validation</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Not separately published in reviewed FTS records</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Provincial response context only</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>No organisation-specific amount identified</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -25698,9 +25850,679 @@
           <t>Technical response partner; local outputs require validation</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Not separately published in reviewed FTS records</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Provincial response context only</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>No organisation-specific amount identified</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="56" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Funding ID</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Operation year</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
+        <is>
+          <t>Funder</t>
+        </is>
+      </c>
+      <c r="D1" s="16" t="inlineStr">
+        <is>
+          <t>Recipient / organisation</t>
+        </is>
+      </c>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>Published amount</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>Currency / amount basis</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>Funding mechanism / status</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>Geographic scope</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>Funding date</t>
+        </is>
+      </c>
+      <c r="J1" s="16" t="inlineStr">
+        <is>
+          <t>Funding QA / local attribution</t>
+        </is>
+      </c>
+      <c r="K1" s="16" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2018-001</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>CERF</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>WHO</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>1,701,255</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>CERF pooled-fund allocation; paid; unearmarked</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri provinces; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>2018-08-23</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed provincial scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A4762&amp;year=2018&amp;boundary=internal&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-001</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>CERF</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>WHO</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>3,902,590</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>CERF pooled-fund allocation; paid; unearmarked</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri provinces; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>2019-09-10</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed provincial scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A4762&amp;year=2019&amp;boundary=internal&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-002</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>CERF</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>1,999,062</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>CERF pooled-fund allocation; paid; unearmarked</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri provinces; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>2019-09-10</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed provincial scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A4762&amp;year=2019&amp;boundary=internal&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-003</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>CERF</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>UNICEF</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>3,935,937</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>CERF pooled-fund allocation; paid; unearmarked</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri provinces; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>2019-09-16</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed provincial scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A4762&amp;year=2019&amp;boundary=internal&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-004</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>European Commission Humanitarian Aid and Civil Protection (ECHO)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>WHO</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>8,476,085</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>USD (original EUR 7,620,000)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>ECHO grant; earmarked; commitment; ref. ECHO/COD/BUD/2019/91025</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri provinces; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>2019-07-04</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed provincial scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A8523&amp;filterBy%5B2%5D=destinationOrganizationId%3A4398&amp;year=2019&amp;boundary=incoming&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-005</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>WHO</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>7,786,429</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>USD (original EUR 7,000,000)</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Government grant; earmarked; commitment; ref. AA-S09 321.50 COD 04/19</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>2019-06-05</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed provincial scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A4306&amp;filterBy%5B2%5D=destinationOrganizationId%3A4398&amp;year=2019&amp;boundary=incoming&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-006</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>European Commission Humanitarian Aid and Civil Protection (ECHO)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>UNICEF</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>889,878</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>USD (original EUR 800,000)</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>ECHO grant; earmarked; paid; ref. ECHO/COD/BUD/2019/91024</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>North Kivu and Ituri; not disaggregated to Mambasa/Mandima</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>2019-06-28</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed provincial scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A8523&amp;filterBy%5B2%5D=destinationOrganizationId%3A2915&amp;year=2019&amp;boundary=incoming&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-007</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Action Against Hunger / ACF</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>538,851</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>USD (original SEK 5,000,000)</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Government grant; earmarked; commitment</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Emergency response to spread of Ebola in Ituri; not disaggregated to Mambasa</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>2019-07-26</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed Ituri scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A2921&amp;filterBy%5B2%5D=destinationOrganizationId%3A4536&amp;year=2019&amp;boundary=incoming&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2019-008</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>European Commission Humanitarian Aid and Civil Protection (ECHO)</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Malteser International</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>888,889</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>USD (original EUR 800,000)</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>ECHO grant; earmarked; commitment; ref. ECHO/COD/BUD/2019/91032</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Northeast Ituri and Haut-Uele; not disaggregated to Mambasa/Watsa/Wamba</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>2019-11-05</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed regional scope; local allocation unavailable</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v1/public/fts/flow?filterBy%5B0%5D=destinationEmergencyId%3A707&amp;filterBy%5B1%5D=sourceOrganizationId%3A8523&amp;filterBy%5B2%5D=destinationOrganizationId%3A173&amp;year=2019&amp;boundary=incoming&amp;report=4&amp;format=json&amp;limit=1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>FND-EB-2026-001</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>OCHA FTS</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>BDBV response</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>0 reported</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>No incoming, outgoing or internal transactions returned in the reviewed FTS query</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>DRC country emergency; no Mambasa/Wamba allocation published</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Source-backed unavailable; zero reported flows do not prove no funding</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>https://api.hpc.tools/v2/public/emergency/id/1031</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>